<commit_message>
Add Naive Bayes, Random Forest, and SVM implementations
- Created Naive Bayes notebook for spam detection using text messages.
- Implemented Random Forest classifier on the Iris dataset with evaluation metrics.
- Added SVM notebook to load and display digit dataset.
</commit_message>
<xml_diff>
--- a/AI_ML_Learnings.xlsx
+++ b/AI_ML_Learnings.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Priya Koma\Desktop\AI_ML\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2031378C-EEEA-4A8F-AFE4-05B1D4C1ED84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C442C969-74C4-443D-B067-91C273956CC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="AI_ML_Beginner" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -509,4 +510,13 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4348CC1-7BEF-4E45-932E-C506D0481A8C}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>